<commit_message>
chore: update checklist data and debug output
- Remove redundant comment annotation in main.py
- Unify checkmark symbol to ✔ in output
- Refresh debug frame content with latest product data
- Update page content debug output
- Update checklist and result Excel files

Auto-commit via auto-git-push
</commit_message>
<xml_diff>
--- a/ai_checker/output/result.xlsx
+++ b/ai_checker/output/result.xlsx
@@ -461,10 +461,14 @@
           <t>SYNCO Wireless Microphone</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SYNCO Wireless Microphone</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -479,10 +483,14 @@
           <t>G4 Pro</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>G4 Pro</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -493,7 +501,11 @@
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>麦克风</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>否</t>
@@ -511,10 +523,14 @@
           <t>SYNCO</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SYNCO</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -529,10 +545,14 @@
           <t>Zhiying Technology</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Zhiying Technology</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -547,10 +567,14 @@
           <t>1.0.0</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -561,7 +585,11 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025/06/17</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>否</t>
@@ -579,10 +607,14 @@
           <t>Microphone/Zhiying Technology/SYNCO/G Series/OpenHarmony-5.1.0.0/G4 Pro/1.0.0/12/version/debug:nolog</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Microphone/Zhiying Technology/SYNCO/G Series/OpenHarmony-5.1.0.0/G4 Pro/1.0.0/12/version/debug:nolog</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -597,10 +629,14 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -615,10 +651,14 @@
           <t>OpenHarmony-5.1.0.0</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>OpenHarmony 5.1.0 Release</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>

</xml_diff>